<commit_message>
feat: export dynamic quote template
</commit_message>
<xml_diff>
--- a/public/templates/bao-gia-nhap-khau-fcl.xlsx
+++ b/public/templates/bao-gia-nhap-khau-fcl.xlsx
@@ -3949,8 +3949,10 @@
       <c r="J7" s="86"/>
     </row>
     <row r="8" spans="1:10" s="3" customFormat="1" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="87" t="s">
-        <v>106</v>
+      <c r="A8" s="87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ngày báo giá: 15/10/2026</t>
+        </is>
       </c>
       <c r="B8" s="87"/>
       <c r="C8" s="87"/>
@@ -3981,7 +3983,11 @@
       <c r="B10" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="C10" s="6"/>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nguyễn Minh (Sales mẫu)</t>
+        </is>
+      </c>
     </row>
     <row r="11" spans="1:10" s="3" customFormat="1" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
@@ -4057,35 +4063,45 @@
       <c r="M17" s="13"/>
     </row>
     <row r="18" spans="1:13" s="3" customFormat="1" ht="27.6" x14ac:dyDescent="0.25">
-      <c r="A18" s="10" t="s">
-        <v>120</v>
-      </c>
-      <c r="B18" s="10" t="s">
-        <v>85</v>
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">333</t>
+        </is>
+      </c>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">33</t>
+        </is>
       </c>
       <c r="C18" s="14">
         <v>1</v>
       </c>
-      <c r="D18" s="10" t="s">
-        <v>98</v>
-      </c>
-      <c r="E18" s="89" t="s">
-        <v>121</v>
+      <c r="D18" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">333</t>
+        </is>
+      </c>
+      <c r="E18" s="89">
+        <v>3231</v>
       </c>
       <c r="F18" s="90"/>
       <c r="G18" s="15">
         <f>E18*C18</f>
-        <v>1450</v>
+        <v>0</v>
       </c>
       <c r="H18" s="16">
         <f>G18*26600</f>
-        <v>38570000</v>
-      </c>
-      <c r="I18" s="17" t="s">
-        <v>124</v>
-      </c>
-      <c r="J18" s="10" t="s">
-        <v>122</v>
+        <v>0</v>
+      </c>
+      <c r="I18" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J18" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="K18" s="13"/>
       <c r="M18" s="18"/>
@@ -4103,8 +4119,10 @@
       <c r="J19" s="19"/>
     </row>
     <row r="20" spans="1:13" s="3" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="9" t="s">
-        <v>91</v>
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2, Xxxx</t>
+        </is>
       </c>
       <c r="B20" s="19"/>
       <c r="C20" s="20"/>
@@ -4119,193 +4137,139 @@
       <c r="J20" s="77"/>
     </row>
     <row r="21" spans="1:13" s="3" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="54" t="s">
-        <v>17</v>
-      </c>
-      <c r="B21" s="55"/>
-      <c r="C21" s="26">
-        <f>C18</f>
-        <v>1</v>
-      </c>
-      <c r="D21" s="10" t="s">
-        <v>37</v>
-      </c>
-      <c r="E21" s="56">
-        <v>250</v>
-      </c>
-      <c r="F21" s="91"/>
-      <c r="G21" s="11">
-        <f>C21*E21</f>
-        <v>250</v>
-      </c>
-      <c r="H21" s="16">
-        <f>G21*26600</f>
-        <v>6650000</v>
-      </c>
-      <c r="I21" s="67"/>
-      <c r="J21" s="67"/>
+      <c r="A21" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Adđ</t>
+        </is>
+      </c>
+      <c r="B21" s="55" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="D21" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dd</t>
+        </is>
+      </c>
+      <c r="E21">
+        <v>322</v>
+      </c>
+      <c r="G21">
+        <f>E21*C21</f>
+        <v>0</v>
+      </c>
+      <c r="H21">
+        <v>2</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="22" spans="1:13" s="3" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="54" t="s">
-        <v>18</v>
-      </c>
-      <c r="B22" s="55"/>
-      <c r="C22" s="23">
-        <f>C21</f>
-        <v>1</v>
-      </c>
-      <c r="D22" s="10" t="s">
-        <v>37</v>
-      </c>
-      <c r="E22" s="56">
-        <v>240</v>
-      </c>
-      <c r="F22" s="91"/>
-      <c r="G22" s="11">
-        <f t="shared" ref="G22:G27" si="0">C22*E22</f>
-        <v>240</v>
-      </c>
-      <c r="H22" s="16">
-        <f t="shared" ref="H22:H27" si="1">G22*26600</f>
-        <v>6384000</v>
-      </c>
-      <c r="I22" s="67"/>
-      <c r="J22" s="67"/>
+      <c r="A22" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3213213</t>
+        </is>
+      </c>
+      <c r="B22" s="55" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="D22" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3123123</t>
+        </is>
+      </c>
+      <c r="E22">
+        <v>0</v>
+      </c>
+      <c r="G22">
+        <f>E22*C22</f>
+        <v>0</v>
+      </c>
+      <c r="H22">
+        <f>G22*26600</f>
+        <v>0</v>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3123</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="23" spans="1:13" s="3" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="54" t="s">
-        <v>38</v>
-      </c>
+      <c r="A23" s="54"/>
       <c r="B23" s="55"/>
-      <c r="C23" s="23">
-        <f>C18</f>
-        <v>1</v>
-      </c>
-      <c r="D23" s="10" t="s">
-        <v>37</v>
-      </c>
-      <c r="E23" s="56">
-        <v>20</v>
-      </c>
+      <c r="D23" s="10"/>
+      <c r="E23" s="56"/>
       <c r="F23" s="91"/>
-      <c r="G23" s="11">
-        <f t="shared" si="0"/>
-        <v>20</v>
-      </c>
-      <c r="H23" s="16">
-        <f t="shared" si="1"/>
-        <v>532000</v>
-      </c>
+      <c r="G23" s="11"/>
+      <c r="H23" s="16"/>
       <c r="I23" s="67"/>
       <c r="J23" s="67"/>
+      <c r="C23"/>
     </row>
     <row r="24" spans="1:13" s="3" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="54" t="s">
-        <v>39</v>
-      </c>
+      <c r="A24" s="54"/>
       <c r="B24" s="55"/>
-      <c r="C24" s="23">
-        <f>C22</f>
-        <v>1</v>
-      </c>
-      <c r="D24" s="10" t="s">
-        <v>37</v>
-      </c>
-      <c r="E24" s="56">
-        <v>20</v>
-      </c>
+      <c r="D24" s="10"/>
+      <c r="E24" s="56"/>
       <c r="F24" s="91"/>
-      <c r="G24" s="11">
-        <f t="shared" si="0"/>
-        <v>20</v>
-      </c>
-      <c r="H24" s="16">
-        <v>500000</v>
-      </c>
+      <c r="G24" s="11"/>
+      <c r="H24" s="16"/>
       <c r="I24" s="67"/>
       <c r="J24" s="67"/>
+      <c r="C24"/>
     </row>
     <row r="25" spans="1:13" s="3" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="54" t="s">
-        <v>19</v>
-      </c>
+      <c r="A25" s="54"/>
       <c r="B25" s="55"/>
-      <c r="C25" s="23">
-        <v>1</v>
-      </c>
-      <c r="D25" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="E25" s="56">
-        <v>35</v>
-      </c>
+      <c r="D25" s="10"/>
+      <c r="E25" s="56"/>
       <c r="F25" s="91"/>
-      <c r="G25" s="11">
-        <f t="shared" si="0"/>
-        <v>35</v>
-      </c>
-      <c r="H25" s="16">
-        <f t="shared" si="1"/>
-        <v>931000</v>
-      </c>
+      <c r="G25" s="11"/>
+      <c r="H25" s="16"/>
       <c r="I25" s="67"/>
       <c r="J25" s="67"/>
+      <c r="C25"/>
     </row>
     <row r="26" spans="1:13" s="3" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="54" t="s">
-        <v>21</v>
-      </c>
+      <c r="A26" s="54"/>
       <c r="B26" s="55"/>
-      <c r="C26" s="23">
-        <v>1</v>
-      </c>
-      <c r="D26" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="E26" s="56">
-        <v>32</v>
-      </c>
+      <c r="D26" s="10"/>
+      <c r="E26" s="56"/>
       <c r="F26" s="57"/>
-      <c r="G26" s="24">
-        <f t="shared" si="0"/>
-        <v>32</v>
-      </c>
-      <c r="H26" s="16">
-        <v>800000</v>
-      </c>
-      <c r="I26" s="58" t="s">
-        <v>126</v>
-      </c>
+      <c r="G26" s="24"/>
+      <c r="H26" s="16"/>
+      <c r="I26" s="58"/>
       <c r="J26" s="59"/>
+      <c r="C26"/>
     </row>
     <row r="27" spans="1:13" s="3" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="54" t="s">
-        <v>123</v>
-      </c>
+      <c r="A27" s="54"/>
       <c r="B27" s="55"/>
-      <c r="C27" s="23">
-        <f>C18</f>
-        <v>1</v>
-      </c>
-      <c r="D27" s="10" t="s">
-        <v>37</v>
-      </c>
-      <c r="E27" s="56">
-        <v>285</v>
-      </c>
+      <c r="D27" s="10"/>
+      <c r="E27" s="56"/>
       <c r="F27" s="57"/>
-      <c r="G27" s="24">
-        <f t="shared" si="0"/>
-        <v>285</v>
-      </c>
-      <c r="H27" s="16">
-        <f t="shared" si="1"/>
-        <v>7581000</v>
-      </c>
-      <c r="I27" s="58" t="s">
-        <v>90</v>
-      </c>
+      <c r="G27" s="24"/>
+      <c r="H27" s="16"/>
+      <c r="I27" s="58"/>
       <c r="J27" s="59"/>
+      <c r="C27"/>
     </row>
     <row r="28" spans="1:13" s="3" customFormat="1" ht="7.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="25"/>
@@ -4332,11 +4296,11 @@
       <c r="F29" s="75"/>
       <c r="G29" s="44">
         <f>SUM(G18:G27)</f>
-        <v>2332</v>
+        <v>0</v>
       </c>
       <c r="H29" s="29">
         <f>SUM(H18:H27)</f>
-        <v>61948000</v>
+        <v>0</v>
       </c>
       <c r="I29" s="76" t="s">
         <v>125</v>

</xml_diff>